<commit_message>
Add the Digital LED load board and align the documentation
- New Hardware/DALI_Load_250W_DigitalLED with the V0.1 fabrication data and
  a Readme covering the connectors, the strip supply and the isolation barrier
- Controller Readme links the two load boards from the actuation paths they
  implement, instead of only describing the options in the abstract
- Root README corrections against the sub-READMEs: Controller is V0.3, the
  bootloader is 1908 / 1920 B, there are 8 output modes (ONOFF was missing),
  and both load boards are listed
- Drop the user-flash size figures from the firmware docs; the boot-area
  figures stay, because that limit is a real constraint
- Refresh the Controller V0.3 and RGBW Gerber exports
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.3).xlsx
+++ b/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.3).xlsx
@@ -1,11 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <bookViews>
-    <workbookView tabRatio="600"/>
-  </bookViews>
   <sheets>
     <sheet name="JLC_PCBA_BOM-DALI_EVG_Controlle" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
@@ -14,442 +11,345 @@
   <definedNames>
     <definedName name="Print_Titles" localSheetId="0">'JLC_PCBA_BOM-DALI_EVG_Controlle'!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="125725" fullPrecision="1"/>
+  <calcPr fullPrecision="1" calcMode="auto" calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="141">
-  <si>
-    <t xml:space="preserve">Comment</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Designator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Footprint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1, C3, C4, C11, C13, C14, C15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C0402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C0603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10uF/50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C12, C19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100nF/50V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C17, C18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">220uF/35V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polarized Capacitor (Axial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAPR-5mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1N4148W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1, D4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOD-123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MB10S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOIC245P670X290-4N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">500mA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F1, F2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GZ1608D601TF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ferrite_Bead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FB1, FB2, FB3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LGS5145</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60-V, 600-mA High Efficiency Wide Input Voltage Range Buck Converter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IC1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT95P280X110-6N (SOT23-6L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C720477</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tactile Switch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J2, J3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS-1088-AR02016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFC 0.5mm 10Pin 90°</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFC 0.5mm 10P Bottom Connection
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="109">
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>Footprint</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>100nF</t>
+  </si>
+  <si>
+    <t>Capacitor</t>
+  </si>
+  <si>
+    <t>C1, C3, C4, C11, C13, C14, C15</t>
+  </si>
+  <si>
+    <t>C0402</t>
+  </si>
+  <si>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>10uF/50V</t>
+  </si>
+  <si>
+    <t>C12, C19</t>
+  </si>
+  <si>
+    <t>C1206</t>
+  </si>
+  <si>
+    <t>100nF/50V</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>C17, C18</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>C21</t>
+  </si>
+  <si>
+    <t>220uF/35V</t>
+  </si>
+  <si>
+    <t>Polarized Capacitor (Axial)</t>
+  </si>
+  <si>
+    <t>C24</t>
+  </si>
+  <si>
+    <t>CAPR-5mm</t>
+  </si>
+  <si>
+    <t>1N4148W</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>D1, D4</t>
+  </si>
+  <si>
+    <t>SOD-123</t>
+  </si>
+  <si>
+    <t>MB10S</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>SOIC245P670X290-4N</t>
+  </si>
+  <si>
+    <t>500mA</t>
+  </si>
+  <si>
+    <t>Fuse</t>
+  </si>
+  <si>
+    <t>F1, F2</t>
+  </si>
+  <si>
+    <t>1206</t>
+  </si>
+  <si>
+    <t>GZ1608D601TF</t>
+  </si>
+  <si>
+    <t>Ferrite_Bead</t>
+  </si>
+  <si>
+    <t>FB1, FB2, FB3</t>
+  </si>
+  <si>
+    <t>0603</t>
+  </si>
+  <si>
+    <t>LGS5145</t>
+  </si>
+  <si>
+    <t>60-V, 600-mA High Efficiency Wide Input Voltage Range Buck Converter</t>
+  </si>
+  <si>
+    <t>IC1</t>
+  </si>
+  <si>
+    <t>SOT95P280X110-6N (SOT23-6L)</t>
+  </si>
+  <si>
+    <t>C720477</t>
+  </si>
+  <si>
+    <t>Tactile Switch</t>
+  </si>
+  <si>
+    <t>J2, J3</t>
+  </si>
+  <si>
+    <t>TS-1088-AR02016</t>
+  </si>
+  <si>
+    <t>FFC 0.5mm 10Pin 90°</t>
+  </si>
+  <si>
+    <t>FFC 0.5mm 10P Bottom Connection
 C262659</t>
   </si>
   <si>
-    <t xml:space="preserve">J4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE_1-1734592-0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminalblock X2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J6, J7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminalblock_X2_5mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMI321609X100KT (10uH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15uH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KF2EDGR-3.5-2Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONN-TH_2P-P3.50_KF2EDGR-3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Header</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 Pin male</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TE_826647-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AO3400A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30V N-Channel MOSFET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT23 Normal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R0805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3, R29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R8, R9, R18, R23, R47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R0603</t>
-  </si>
-  <si>
-    <t xml:space="preserve">470k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.7k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.2k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CH32V003F4U6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LMV331IDBVRG4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT23-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AT24C256C-SSHL-T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOIC127P600X265-8N (SOIC-8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JLCPCB Part #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C307331</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1588</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C13585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C59461</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C15849</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C81598</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2488</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C99561</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5123971</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C262659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C474881</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C441171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C20917</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25271</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C11702</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25741</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25744</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25756</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C22859</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C23178</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C23162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25981</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25810</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4216</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5299908</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C34731</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C6482</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1590097</t>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>TE_1-1734592-0</t>
+  </si>
+  <si>
+    <t>Terminalblock X2</t>
+  </si>
+  <si>
+    <t>J6, J7</t>
+  </si>
+  <si>
+    <t>Terminalblock_X2_5mm</t>
+  </si>
+  <si>
+    <t>CMI321609X100KT (10uH)</t>
+  </si>
+  <si>
+    <t>15uH</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L1210</t>
+  </si>
+  <si>
+    <t>KF2EDGR-3.5-2Pin</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>CONN-TH_2P-P3.50_KF2EDGR-3.5</t>
+  </si>
+  <si>
+    <t>Header</t>
+  </si>
+  <si>
+    <t>4 Pin male</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>TE_826647-4</t>
+  </si>
+  <si>
+    <t>AO3400A</t>
+  </si>
+  <si>
+    <t>30V N-Channel MOSFET</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>SOT23 Normal</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R0805</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>R3, R29</t>
+  </si>
+  <si>
+    <t>0402</t>
+  </si>
+  <si>
+    <t>100k</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>R8, R9, R18, R23, R47</t>
+  </si>
+  <si>
+    <t>15k</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>R27</t>
+  </si>
+  <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>470k</t>
+  </si>
+  <si>
+    <t>R28</t>
+  </si>
+  <si>
+    <t>4.7k</t>
+  </si>
+  <si>
+    <t>R30</t>
+  </si>
+  <si>
+    <t>R31</t>
+  </si>
+  <si>
+    <t>8.2k</t>
+  </si>
+  <si>
+    <t>R32</t>
+  </si>
+  <si>
+    <t>18k</t>
+  </si>
+  <si>
+    <t>R33</t>
+  </si>
+  <si>
+    <t>33k</t>
+  </si>
+  <si>
+    <t>R46</t>
+  </si>
+  <si>
+    <t>CH32V003F4U6</t>
+  </si>
+  <si>
+    <t>CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
+  </si>
+  <si>
+    <t>LMV331IDBVRG4</t>
+  </si>
+  <si>
+    <t>Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>SOT23-5</t>
+  </si>
+  <si>
+    <t>AT24C256C-SSHL-T</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>SOIC127P600X265-8N (SOIC-8)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <fonts count="5">
     <font>
       <sz val="10"/>
@@ -651,68 +551,68 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="42" fontId="1" fillId="2" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="2" borderId="0"/>
+  <cellStyleXfs count="6">
+    <xf xxid="0" numFmtId="0" fontId="0" fillId="2" borderId="0"/>
+    <xf xxid="1" numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="2" numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="3" numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="4" numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="5" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="6" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="7" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="8" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="9" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="10" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="11" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="12" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="13" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="14" numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="16" numFmtId="43" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="17" numFmtId="41" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="18" numFmtId="44" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="19" numFmtId="42" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf xxid="20" numFmtId="9" fontId="1" fillId="2" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+  <cellXfs>
+    <xf xxid="15" numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
+    <xf xxid="21" numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf xxid="22" numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf xxid="23" numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyBorder="1"/>
+    <xf xxid="24" numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyBorder="1"/>
+    <xf xxid="25" numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyBorder="1"/>
+    <xf xxid="26" numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1"/>
+    <xf xxid="27" numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1"/>
+    <xf xxid="28" numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1"/>
+    <xf xxid="29" numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1"/>
+    <xf xxid="30" numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyBorder="1"/>
+    <xf xxid="31" numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyBorder="1"/>
+    <xf xxid="32" numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyBorder="1"/>
+    <xf xxid="33" numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyBorder="1"/>
+    <xf xxid="34" numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyBorder="1" applyFill="1"/>
+    <xf xxid="35" numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyBorder="1" applyFill="1"/>
+    <xf xxid="36" numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="37" numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="38" numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" quotePrefix="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf xxid="39" numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyAlignment="1" applyBorder="1" quotePrefix="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf xxid="40" numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyBorder="1"/>
+    <xf xxid="41" numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="42" numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="43" numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyBorder="1"/>
+    <xf xxid="44" numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyBorder="1"/>
+    <xf xxid="45" numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="46" numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="47" numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyBorder="1"/>
+    <xf xxid="48" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="49" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="50" numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyBorder="1"/>
+    <xf xxid="51" numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyBorder="1" applyFill="1"/>
+    <xf xxid="52" numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyBorder="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -722,15 +622,15 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="" defaultPivotStyle=""/>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="A1:F35"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr defaultRowHeight="12.75" baseColWidth="0"/>
   <cols>
     <col min="1" max="5" width="20.2109375" customWidth="1"/>
   </cols>
@@ -751,9 +651,6 @@
       <c r="E1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="32" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="26" t="s">
@@ -771,9 +668,6 @@
       <c r="E2" s="27">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>110</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="29" t="s">
@@ -791,9 +685,6 @@
       <c r="E3" s="30">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="29" t="s">
@@ -811,9 +702,6 @@
       <c r="E4" s="30">
         <v>2</v>
       </c>
-      <c r="F4" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="29" t="s">
@@ -831,9 +719,6 @@
       <c r="E5" s="30">
         <v>1</v>
       </c>
-      <c r="F5" t="s">
-        <v>110</v>
-      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="29" t="s">
@@ -851,9 +736,6 @@
       <c r="E6" s="30">
         <v>2</v>
       </c>
-      <c r="F6" t="s">
-        <v>113</v>
-      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="29" t="s">
@@ -871,9 +753,6 @@
       <c r="E7" s="30">
         <v>1</v>
       </c>
-      <c r="F7" t="s">
-        <v>114</v>
-      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="29" t="s">
@@ -891,9 +770,6 @@
       <c r="E8" s="30">
         <v>1</v>
       </c>
-      <c r="F8" t="s">
-        <v>140</v>
-      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="29" t="s">
@@ -911,9 +787,6 @@
       <c r="E9" s="30">
         <v>2</v>
       </c>
-      <c r="F9" t="s">
-        <v>115</v>
-      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="29" t="s">
@@ -931,9 +804,6 @@
       <c r="E10" s="30">
         <v>1</v>
       </c>
-      <c r="F10" t="s">
-        <v>116</v>
-      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="29" t="s">
@@ -951,9 +821,6 @@
       <c r="E11" s="30">
         <v>2</v>
       </c>
-      <c r="F11" t="s">
-        <v>117</v>
-      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="29" t="s">
@@ -971,9 +838,6 @@
       <c r="E12" s="30">
         <v>3</v>
       </c>
-      <c r="F12" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="29" t="s">
@@ -991,9 +855,6 @@
       <c r="E13" s="30">
         <v>1</v>
       </c>
-      <c r="F13" t="s">
-        <v>119</v>
-      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="29" t="s">
@@ -1011,9 +872,6 @@
       <c r="E14" s="30">
         <v>2</v>
       </c>
-      <c r="F14" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="29" t="s">
@@ -1031,9 +889,6 @@
       <c r="E15" s="30">
         <v>1</v>
       </c>
-      <c r="F15" t="s">
-        <v>120</v>
-      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="29" t="s">
@@ -1051,9 +906,6 @@
       <c r="E16" s="30">
         <v>2</v>
       </c>
-      <c r="F16" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="29" t="s">
@@ -1071,9 +923,6 @@
       <c r="E17" s="30">
         <v>1</v>
       </c>
-      <c r="F17" t="s">
-        <v>122</v>
-      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="29" t="s">
@@ -1091,9 +940,6 @@
       <c r="E18" s="30">
         <v>1</v>
       </c>
-      <c r="F18" t="s">
-        <v>123</v>
-      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="29" t="s">
@@ -1128,9 +974,6 @@
       <c r="E20" s="30">
         <v>1</v>
       </c>
-      <c r="F20" t="s">
-        <v>124</v>
-      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="29" t="s">
@@ -1148,9 +991,6 @@
       <c r="E21" s="30">
         <v>1</v>
       </c>
-      <c r="F21" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="29" t="s">
@@ -1168,9 +1008,6 @@
       <c r="E22" s="30">
         <v>2</v>
       </c>
-      <c r="F22" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="29" t="s">
@@ -1188,9 +1025,6 @@
       <c r="E23" s="30">
         <v>1</v>
       </c>
-      <c r="F23" t="s">
-        <v>127</v>
-      </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="29" t="s">
@@ -1208,9 +1042,6 @@
       <c r="E24" s="30">
         <v>5</v>
       </c>
-      <c r="F24" t="s">
-        <v>128</v>
-      </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="29" t="s">
@@ -1228,9 +1059,6 @@
       <c r="E25" s="30">
         <v>1</v>
       </c>
-      <c r="F25" t="s">
-        <v>129</v>
-      </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="29" t="s">
@@ -1248,9 +1076,6 @@
       <c r="E26" s="30">
         <v>1</v>
       </c>
-      <c r="F26" t="s">
-        <v>130</v>
-      </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="29" t="s">
@@ -1268,9 +1093,6 @@
       <c r="E27" s="30">
         <v>1</v>
       </c>
-      <c r="F27" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="29" t="s">
@@ -1288,9 +1110,6 @@
       <c r="E28" s="30">
         <v>1</v>
       </c>
-      <c r="F28" t="s">
-        <v>132</v>
-      </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="29" t="s">
@@ -1308,9 +1127,6 @@
       <c r="E29" s="30">
         <v>1</v>
       </c>
-      <c r="F29" t="s">
-        <v>133</v>
-      </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="29" t="s">
@@ -1328,9 +1144,6 @@
       <c r="E30" s="30">
         <v>1</v>
       </c>
-      <c r="F30" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="29" t="s">
@@ -1348,9 +1161,6 @@
       <c r="E31" s="30">
         <v>1</v>
       </c>
-      <c r="F31" t="s">
-        <v>135</v>
-      </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="29" t="s">
@@ -1368,9 +1178,6 @@
       <c r="E32" s="30">
         <v>1</v>
       </c>
-      <c r="F32" t="s">
-        <v>136</v>
-      </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="29" t="s">
@@ -1388,9 +1195,6 @@
       <c r="E33" s="30">
         <v>1</v>
       </c>
-      <c r="F33" t="s">
-        <v>137</v>
-      </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="29" t="s">
@@ -1408,9 +1212,6 @@
       <c r="E34" s="30">
         <v>1</v>
       </c>
-      <c r="F34" t="s">
-        <v>138</v>
-      </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="29" t="s">
@@ -1427,9 +1228,6 @@
       </c>
       <c r="E35" s="30">
         <v>1</v>
-      </c>
-      <c r="F35" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>